<commit_message>
Atualiza produtos e suaviza capa do portfolio
</commit_message>
<xml_diff>
--- a/dados/produtos_catalogo.xlsx
+++ b/dados/produtos_catalogo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://infostore-my.sharepoint.com/personal/ana_santos_infostore_com_br/Documents/Área de Trabalho/clubone-catalogo/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_84C5441E015BB5BB910775DDC721F807AB5255A6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F67AC01-6F9F-4850-8E59-D266A65B623B}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_84C5441E015BB5BB910775DDC721F807AB5255A6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0864D4AD-0636-4D6A-B927-8802F72E4AA1}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="4725" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1121" uniqueCount="687">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="725">
   <si>
     <t>FABRICANTE</t>
   </si>
@@ -2094,6 +2094,120 @@
   </si>
   <si>
     <t>HR1501</t>
+  </si>
+  <si>
+    <t>ADE0002</t>
+  </si>
+  <si>
+    <t>ADEGA 12 GARRAFAS ACB12 PRE 127V</t>
+  </si>
+  <si>
+    <t>01121WBA089</t>
+  </si>
+  <si>
+    <t>FOG0051</t>
+  </si>
+  <si>
+    <t>COOKTOP 5 BOCAS GAS KE5HP HOME PRO PRE BIV (TRIPLA</t>
+  </si>
+  <si>
+    <t>66809HBA088</t>
+  </si>
+  <si>
+    <t>FOG0055</t>
+  </si>
+  <si>
+    <t>COOKTOP 5 BOCAS GAS KE5PS PRO SERIES BIVOLT</t>
+  </si>
+  <si>
+    <t>66809PBA035</t>
+  </si>
+  <si>
+    <t>FOG0065</t>
+  </si>
+  <si>
+    <t>FOG  4 BOCAS EFFIC FE4GB PRE BIVOLT (M.VID)</t>
+  </si>
+  <si>
+    <t>63041VBA035</t>
+  </si>
+  <si>
+    <t>FOG0068</t>
+  </si>
+  <si>
+    <t>FOG  4 BOCAS EFFIC FE4IG CIN BIVOLT (M.VID)</t>
+  </si>
+  <si>
+    <t>23041IBA088</t>
+  </si>
+  <si>
+    <t>GEL0111</t>
+  </si>
+  <si>
+    <t>GELADEIRA FF 380L DUPLEX IF41S CIN 127V</t>
+  </si>
+  <si>
+    <t>02353FBA130</t>
+  </si>
+  <si>
+    <t>GEL0112</t>
+  </si>
+  <si>
+    <t>GELADEIRA FF 380L DUPLEX IF41 BRA 127V</t>
+  </si>
+  <si>
+    <t>02352FBA106</t>
+  </si>
+  <si>
+    <t>LAV0027</t>
+  </si>
+  <si>
+    <t>MAQ LAV  TL   9KG LED09 BRA 127V</t>
+  </si>
+  <si>
+    <t>2109CDBA106</t>
+  </si>
+  <si>
+    <t>LAV0052</t>
+  </si>
+  <si>
+    <t>MAQ LAV  TL 18KG LEB18 PRE 127V (CESTINOX)</t>
+  </si>
+  <si>
+    <t>2118CDBB135</t>
+  </si>
+  <si>
+    <t>LAV0056</t>
+  </si>
+  <si>
+    <t>MAQ LAV  TL 14,5KG LEE15 BRA 127V (CESTINOX)</t>
+  </si>
+  <si>
+    <t>LAV0061</t>
+  </si>
+  <si>
+    <t>LAVA  E SECA INV 12KG LSC12 CIN 127V</t>
+  </si>
+  <si>
+    <t>5112QDBA199</t>
+  </si>
+  <si>
+    <t>LAV0062</t>
+  </si>
+  <si>
+    <t>MAQ LAV FL 12KG INV 12KG LFC12 CIN 127V</t>
+  </si>
+  <si>
+    <t>1512QDBA199</t>
+  </si>
+  <si>
+    <t>MIC0009</t>
+  </si>
+  <si>
+    <t>MICRO-ONDAS EMBUTIR 34L EXPERIENCE ME3EP PRE 127V</t>
+  </si>
+  <si>
+    <t>10341CBA135</t>
   </si>
 </sst>
 </file>
@@ -2162,8 +2276,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tb_produtos" displayName="tb_produtos" ref="A1:L223" totalsRowShown="0">
-  <autoFilter ref="A1:L223" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tb_produtos" displayName="tb_produtos" ref="A1:L236" totalsRowShown="0">
+  <autoFilter ref="A1:L236" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="FABRICANTE"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="SEGMENTO"/>
@@ -2377,7 +2491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L223"/>
+  <dimension ref="A1:L236"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -6207,6 +6321,227 @@
         <v>669</v>
       </c>
     </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A224" t="s">
+        <v>211</v>
+      </c>
+      <c r="B224" t="s">
+        <v>106</v>
+      </c>
+      <c r="C224" t="s">
+        <v>687</v>
+      </c>
+      <c r="D224" t="s">
+        <v>688</v>
+      </c>
+      <c r="E224" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A225" t="s">
+        <v>211</v>
+      </c>
+      <c r="B225" t="s">
+        <v>106</v>
+      </c>
+      <c r="C225" t="s">
+        <v>690</v>
+      </c>
+      <c r="D225" t="s">
+        <v>691</v>
+      </c>
+      <c r="E225" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A226" t="s">
+        <v>211</v>
+      </c>
+      <c r="B226" t="s">
+        <v>106</v>
+      </c>
+      <c r="C226" t="s">
+        <v>693</v>
+      </c>
+      <c r="D226" t="s">
+        <v>694</v>
+      </c>
+      <c r="E226" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A227" t="s">
+        <v>211</v>
+      </c>
+      <c r="B227" t="s">
+        <v>106</v>
+      </c>
+      <c r="C227" t="s">
+        <v>696</v>
+      </c>
+      <c r="D227" t="s">
+        <v>697</v>
+      </c>
+      <c r="E227" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A228" t="s">
+        <v>211</v>
+      </c>
+      <c r="B228" t="s">
+        <v>106</v>
+      </c>
+      <c r="C228" t="s">
+        <v>699</v>
+      </c>
+      <c r="D228" t="s">
+        <v>700</v>
+      </c>
+      <c r="E228" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A229" t="s">
+        <v>211</v>
+      </c>
+      <c r="B229" t="s">
+        <v>106</v>
+      </c>
+      <c r="C229" t="s">
+        <v>702</v>
+      </c>
+      <c r="D229" t="s">
+        <v>703</v>
+      </c>
+      <c r="E229" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A230" t="s">
+        <v>211</v>
+      </c>
+      <c r="B230" t="s">
+        <v>106</v>
+      </c>
+      <c r="C230" t="s">
+        <v>705</v>
+      </c>
+      <c r="D230" t="s">
+        <v>706</v>
+      </c>
+      <c r="E230" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A231" t="s">
+        <v>211</v>
+      </c>
+      <c r="B231" t="s">
+        <v>106</v>
+      </c>
+      <c r="C231" t="s">
+        <v>708</v>
+      </c>
+      <c r="D231" t="s">
+        <v>709</v>
+      </c>
+      <c r="E231" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A232" t="s">
+        <v>211</v>
+      </c>
+      <c r="B232" t="s">
+        <v>106</v>
+      </c>
+      <c r="C232" t="s">
+        <v>711</v>
+      </c>
+      <c r="D232" t="s">
+        <v>712</v>
+      </c>
+      <c r="E232" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A233" t="s">
+        <v>211</v>
+      </c>
+      <c r="B233" t="s">
+        <v>106</v>
+      </c>
+      <c r="C233" t="s">
+        <v>714</v>
+      </c>
+      <c r="D233" t="s">
+        <v>715</v>
+      </c>
+      <c r="E233" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A234" t="s">
+        <v>211</v>
+      </c>
+      <c r="B234" t="s">
+        <v>106</v>
+      </c>
+      <c r="C234" t="s">
+        <v>716</v>
+      </c>
+      <c r="D234" t="s">
+        <v>717</v>
+      </c>
+      <c r="E234" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A235" t="s">
+        <v>211</v>
+      </c>
+      <c r="B235" t="s">
+        <v>106</v>
+      </c>
+      <c r="C235" t="s">
+        <v>719</v>
+      </c>
+      <c r="D235" t="s">
+        <v>720</v>
+      </c>
+      <c r="E235" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A236" t="s">
+        <v>211</v>
+      </c>
+      <c r="B236" t="s">
+        <v>106</v>
+      </c>
+      <c r="C236" t="s">
+        <v>722</v>
+      </c>
+      <c r="D236" t="s">
+        <v>723</v>
+      </c>
+      <c r="E236" t="s">
+        <v>724</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Atualiza catalogo com JBL, imagens e enriquecimento
</commit_message>
<xml_diff>
--- a/dados/produtos_catalogo.xlsx
+++ b/dados/produtos_catalogo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://infostore-my.sharepoint.com/personal/ana_santos_infostore_com_br/Documents/Área de Trabalho/clubone-catalogo/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_84C5441E015BB5BB910775DDC721F807AB5255A6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0864D4AD-0636-4D6A-B927-8802F72E4AA1}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_84C5441E015BB5BB910775DDC721F807AB5255A6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A83634B9-6543-484E-B1FE-02B5E265CB5A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="4725" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="725">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1216" uniqueCount="745">
   <si>
     <t>FABRICANTE</t>
   </si>
@@ -2208,6 +2208,66 @@
   </si>
   <si>
     <t>10341CBA135</t>
+  </si>
+  <si>
+    <t>JBL (NAC)</t>
+  </si>
+  <si>
+    <t>AUDIO</t>
+  </si>
+  <si>
+    <t>HOM0167</t>
+  </si>
+  <si>
+    <t>SOUNDBAR  7.1.4 BAR 1000 MULTIBEAM (440W/WIF/BT)</t>
+  </si>
+  <si>
+    <t>28913595</t>
+  </si>
+  <si>
+    <t>HOM0168</t>
+  </si>
+  <si>
+    <t>SOUNDBAR 11.1.4 BAR 1300X MULTIBEAM (585W/WIF/BT)</t>
+  </si>
+  <si>
+    <t>28913658</t>
+  </si>
+  <si>
+    <t>HOM0212</t>
+  </si>
+  <si>
+    <t>SOUNDBAR  5.1 BAR 500MK2 MULTIBEAM (375W/BT/2HDMI/OPT</t>
+  </si>
+  <si>
+    <t>28913881</t>
+  </si>
+  <si>
+    <t>HOM0213</t>
+  </si>
+  <si>
+    <t>SOUNDBAR  7.1.4 BAR 1000MK2 MULTIBEAM (480W/BT/4HDMI/OPT)</t>
+  </si>
+  <si>
+    <t>28913884</t>
+  </si>
+  <si>
+    <t>HOM0214</t>
+  </si>
+  <si>
+    <t>SOUNDBAR  7.1 BAR 800MK2 MULTIBEAM (390W/BT/2HDMI/OPT</t>
+  </si>
+  <si>
+    <t>28913883</t>
+  </si>
+  <si>
+    <t>HOM0215</t>
+  </si>
+  <si>
+    <t>SOUNDBAR 11.1.4 BAR 1300XMK2 MULTIBEAM (785W/BT/3HDMI/OPT</t>
+  </si>
+  <si>
+    <t>28913885</t>
   </si>
 </sst>
 </file>
@@ -2491,7 +2551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L236"/>
+  <dimension ref="A1:L242"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -6542,6 +6602,108 @@
         <v>724</v>
       </c>
     </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A237" t="s">
+        <v>725</v>
+      </c>
+      <c r="B237" t="s">
+        <v>726</v>
+      </c>
+      <c r="C237" t="s">
+        <v>733</v>
+      </c>
+      <c r="D237" t="s">
+        <v>734</v>
+      </c>
+      <c r="E237" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A238" t="s">
+        <v>725</v>
+      </c>
+      <c r="B238" t="s">
+        <v>726</v>
+      </c>
+      <c r="C238" t="s">
+        <v>736</v>
+      </c>
+      <c r="D238" t="s">
+        <v>737</v>
+      </c>
+      <c r="E238" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A239" t="s">
+        <v>725</v>
+      </c>
+      <c r="B239" t="s">
+        <v>726</v>
+      </c>
+      <c r="C239" t="s">
+        <v>739</v>
+      </c>
+      <c r="D239" t="s">
+        <v>740</v>
+      </c>
+      <c r="E239" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A240" t="s">
+        <v>725</v>
+      </c>
+      <c r="B240" t="s">
+        <v>726</v>
+      </c>
+      <c r="C240" t="s">
+        <v>742</v>
+      </c>
+      <c r="D240" t="s">
+        <v>743</v>
+      </c>
+      <c r="E240" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A241" t="s">
+        <v>725</v>
+      </c>
+      <c r="B241" t="s">
+        <v>726</v>
+      </c>
+      <c r="C241" t="s">
+        <v>727</v>
+      </c>
+      <c r="D241" t="s">
+        <v>728</v>
+      </c>
+      <c r="E241" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A242" t="s">
+        <v>725</v>
+      </c>
+      <c r="B242" t="s">
+        <v>726</v>
+      </c>
+      <c r="C242" t="s">
+        <v>730</v>
+      </c>
+      <c r="D242" t="s">
+        <v>731</v>
+      </c>
+      <c r="E242" t="s">
+        <v>732</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>